<commit_message>
fix: keep asset department linked to assignee
</commit_message>
<xml_diff>
--- a/backend/assets/data/资产导入模板.xlsx
+++ b/backend/assets/data/资产导入模板.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资产导入" sheetId="1" r:id="Rf751cfae26084af2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="R05b6d32946ca463d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资产导入" sheetId="1" r:id="R6c5a72bd79f34b1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="Rcfd72a3e3e62422e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -316,6 +316,32 @@
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AssetImportTable" displayName="AssetImportTable" ref="A1:R101" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="18">
+    <x:tableColumn id="1" name="资产分类"/>
+    <x:tableColumn id="2" name="资产类型"/>
+    <x:tableColumn id="3" name="金蝶编码"/>
+    <x:tableColumn id="4" name="责任人"/>
+    <x:tableColumn id="5" name="状态"/>
+    <x:tableColumn id="6" name="资产位置"/>
+    <x:tableColumn id="7" name="品牌"/>
+    <x:tableColumn id="8" name="型号"/>
+    <x:tableColumn id="9" name="数量"/>
+    <x:tableColumn id="10" name="设备序列号"/>
+    <x:tableColumn id="11" name="规格配置"/>
+    <x:tableColumn id="12" name="CPU"/>
+    <x:tableColumn id="13" name="硬盘大小(G)"/>
+    <x:tableColumn id="14" name="内存(G)"/>
+    <x:tableColumn id="15" name="有线MAC地址"/>
+    <x:tableColumn id="16" name="无线MAC地址"/>
+    <x:tableColumn id="17" name="购买日期"/>
+    <x:tableColumn id="18" name="备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -518,19 +544,19 @@
     <x:col min="3" max="3" width="17" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="17" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="9" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="22" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="28" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="15" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="13" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="9" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="28" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="15" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="13" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="20" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="20" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="20" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="16" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="16" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="30" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="30" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -551,47 +577,45 @@
         <x:v>状态</x:v>
       </x:c>
       <x:c r="F1" s="13" t="str">
-        <x:v>部门</x:v>
+        <x:v>资产位置</x:v>
       </x:c>
       <x:c r="G1" s="13" t="str">
-        <x:v>资产位置</x:v>
+        <x:v>品牌</x:v>
       </x:c>
       <x:c r="H1" s="13" t="str">
-        <x:v>品牌</x:v>
+        <x:v>型号</x:v>
       </x:c>
       <x:c r="I1" s="13" t="str">
-        <x:v>型号</x:v>
+        <x:v>数量</x:v>
       </x:c>
       <x:c r="J1" s="13" t="str">
-        <x:v>数量</x:v>
+        <x:v>设备序列号</x:v>
       </x:c>
       <x:c r="K1" s="13" t="str">
-        <x:v>设备序列号</x:v>
+        <x:v>规格配置</x:v>
       </x:c>
       <x:c r="L1" s="13" t="str">
-        <x:v>规格配置</x:v>
+        <x:v>CPU</x:v>
       </x:c>
       <x:c r="M1" s="13" t="str">
-        <x:v>CPU</x:v>
+        <x:v>硬盘大小(G)</x:v>
       </x:c>
       <x:c r="N1" s="13" t="str">
-        <x:v>硬盘大小(G)</x:v>
+        <x:v>内存(G)</x:v>
       </x:c>
       <x:c r="O1" s="13" t="str">
-        <x:v>内存(G)</x:v>
+        <x:v>有线MAC地址</x:v>
       </x:c>
       <x:c r="P1" s="13" t="str">
-        <x:v>有线MAC地址</x:v>
+        <x:v>无线MAC地址</x:v>
       </x:c>
       <x:c r="Q1" s="13" t="str">
-        <x:v>无线MAC地址</x:v>
+        <x:v>购买日期</x:v>
       </x:c>
       <x:c r="R1" s="13" t="str">
-        <x:v>购买日期</x:v>
-      </x:c>
-      <x:c r="S1" s="14" t="str">
         <x:v>备注</x:v>
       </x:c>
+      <x:c r="S1"/>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="23"/>
@@ -612,7 +636,7 @@
       <x:c r="P2" s="26"/>
       <x:c r="Q2" s="26"/>
       <x:c r="R2" s="32"/>
-      <x:c r="S2" s="20"/>
+      <x:c r="S2"/>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="24"/>
@@ -633,7 +657,7 @@
       <x:c r="P3" s="27"/>
       <x:c r="Q3" s="27"/>
       <x:c r="R3" s="33"/>
-      <x:c r="S3" s="21"/>
+      <x:c r="S3"/>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="24"/>
@@ -654,7 +678,7 @@
       <x:c r="P4" s="27"/>
       <x:c r="Q4" s="27"/>
       <x:c r="R4" s="33"/>
-      <x:c r="S4" s="21"/>
+      <x:c r="S4"/>
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="24"/>
@@ -675,7 +699,7 @@
       <x:c r="P5" s="27"/>
       <x:c r="Q5" s="27"/>
       <x:c r="R5" s="33"/>
-      <x:c r="S5" s="21"/>
+      <x:c r="S5"/>
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="24"/>
@@ -696,7 +720,7 @@
       <x:c r="P6" s="27"/>
       <x:c r="Q6" s="27"/>
       <x:c r="R6" s="33"/>
-      <x:c r="S6" s="21"/>
+      <x:c r="S6"/>
     </x:row>
     <x:row r="7" ht="24" customHeight="1">
       <x:c r="A7" s="24"/>
@@ -717,7 +741,7 @@
       <x:c r="P7" s="27"/>
       <x:c r="Q7" s="27"/>
       <x:c r="R7" s="33"/>
-      <x:c r="S7" s="21"/>
+      <x:c r="S7"/>
     </x:row>
     <x:row r="8" ht="24" customHeight="1">
       <x:c r="A8" s="24"/>
@@ -738,7 +762,7 @@
       <x:c r="P8" s="27"/>
       <x:c r="Q8" s="27"/>
       <x:c r="R8" s="33"/>
-      <x:c r="S8" s="21"/>
+      <x:c r="S8"/>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
       <x:c r="A9" s="24"/>
@@ -759,7 +783,7 @@
       <x:c r="P9" s="27"/>
       <x:c r="Q9" s="27"/>
       <x:c r="R9" s="33"/>
-      <x:c r="S9" s="21"/>
+      <x:c r="S9"/>
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
       <x:c r="A10" s="24"/>
@@ -780,7 +804,7 @@
       <x:c r="P10" s="27"/>
       <x:c r="Q10" s="27"/>
       <x:c r="R10" s="33"/>
-      <x:c r="S10" s="21"/>
+      <x:c r="S10"/>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
       <x:c r="A11" s="24"/>
@@ -801,7 +825,7 @@
       <x:c r="P11" s="27"/>
       <x:c r="Q11" s="27"/>
       <x:c r="R11" s="33"/>
-      <x:c r="S11" s="21"/>
+      <x:c r="S11"/>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
       <x:c r="A12" s="24"/>
@@ -822,7 +846,7 @@
       <x:c r="P12" s="27"/>
       <x:c r="Q12" s="27"/>
       <x:c r="R12" s="33"/>
-      <x:c r="S12" s="21"/>
+      <x:c r="S12"/>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
       <x:c r="A13" s="24"/>
@@ -843,7 +867,7 @@
       <x:c r="P13" s="27"/>
       <x:c r="Q13" s="27"/>
       <x:c r="R13" s="33"/>
-      <x:c r="S13" s="21"/>
+      <x:c r="S13"/>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
       <x:c r="A14" s="24"/>
@@ -864,7 +888,7 @@
       <x:c r="P14" s="27"/>
       <x:c r="Q14" s="27"/>
       <x:c r="R14" s="33"/>
-      <x:c r="S14" s="21"/>
+      <x:c r="S14"/>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="24"/>
@@ -885,7 +909,7 @@
       <x:c r="P15" s="27"/>
       <x:c r="Q15" s="27"/>
       <x:c r="R15" s="33"/>
-      <x:c r="S15" s="21"/>
+      <x:c r="S15"/>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
       <x:c r="A16" s="24"/>
@@ -906,7 +930,7 @@
       <x:c r="P16" s="27"/>
       <x:c r="Q16" s="27"/>
       <x:c r="R16" s="33"/>
-      <x:c r="S16" s="21"/>
+      <x:c r="S16"/>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
       <x:c r="A17" s="24"/>
@@ -927,7 +951,7 @@
       <x:c r="P17" s="27"/>
       <x:c r="Q17" s="27"/>
       <x:c r="R17" s="33"/>
-      <x:c r="S17" s="21"/>
+      <x:c r="S17"/>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
       <x:c r="A18" s="24"/>
@@ -948,7 +972,7 @@
       <x:c r="P18" s="27"/>
       <x:c r="Q18" s="27"/>
       <x:c r="R18" s="33"/>
-      <x:c r="S18" s="21"/>
+      <x:c r="S18"/>
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
       <x:c r="A19" s="24"/>
@@ -969,7 +993,7 @@
       <x:c r="P19" s="27"/>
       <x:c r="Q19" s="27"/>
       <x:c r="R19" s="33"/>
-      <x:c r="S19" s="21"/>
+      <x:c r="S19"/>
     </x:row>
     <x:row r="20" ht="24" customHeight="1">
       <x:c r="A20" s="24"/>
@@ -990,7 +1014,7 @@
       <x:c r="P20" s="27"/>
       <x:c r="Q20" s="27"/>
       <x:c r="R20" s="33"/>
-      <x:c r="S20" s="21"/>
+      <x:c r="S20"/>
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="24"/>
@@ -1011,7 +1035,7 @@
       <x:c r="P21" s="27"/>
       <x:c r="Q21" s="27"/>
       <x:c r="R21" s="33"/>
-      <x:c r="S21" s="21"/>
+      <x:c r="S21"/>
     </x:row>
     <x:row r="22" ht="24" customHeight="1">
       <x:c r="A22" s="24"/>
@@ -1032,7 +1056,7 @@
       <x:c r="P22" s="27"/>
       <x:c r="Q22" s="27"/>
       <x:c r="R22" s="33"/>
-      <x:c r="S22" s="21"/>
+      <x:c r="S22"/>
     </x:row>
     <x:row r="23" ht="24" customHeight="1">
       <x:c r="A23" s="24"/>
@@ -1053,7 +1077,7 @@
       <x:c r="P23" s="27"/>
       <x:c r="Q23" s="27"/>
       <x:c r="R23" s="33"/>
-      <x:c r="S23" s="21"/>
+      <x:c r="S23"/>
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="24"/>
@@ -1074,7 +1098,7 @@
       <x:c r="P24" s="27"/>
       <x:c r="Q24" s="27"/>
       <x:c r="R24" s="33"/>
-      <x:c r="S24" s="21"/>
+      <x:c r="S24"/>
     </x:row>
     <x:row r="25" ht="24" customHeight="1">
       <x:c r="A25" s="24"/>
@@ -1095,7 +1119,7 @@
       <x:c r="P25" s="27"/>
       <x:c r="Q25" s="27"/>
       <x:c r="R25" s="33"/>
-      <x:c r="S25" s="21"/>
+      <x:c r="S25"/>
     </x:row>
     <x:row r="26" ht="24" customHeight="1">
       <x:c r="A26" s="24"/>
@@ -1116,7 +1140,7 @@
       <x:c r="P26" s="27"/>
       <x:c r="Q26" s="27"/>
       <x:c r="R26" s="33"/>
-      <x:c r="S26" s="21"/>
+      <x:c r="S26"/>
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
       <x:c r="A27" s="24"/>
@@ -1137,7 +1161,7 @@
       <x:c r="P27" s="27"/>
       <x:c r="Q27" s="27"/>
       <x:c r="R27" s="33"/>
-      <x:c r="S27" s="21"/>
+      <x:c r="S27"/>
     </x:row>
     <x:row r="28" ht="24" customHeight="1">
       <x:c r="A28" s="24"/>
@@ -1158,7 +1182,7 @@
       <x:c r="P28" s="27"/>
       <x:c r="Q28" s="27"/>
       <x:c r="R28" s="33"/>
-      <x:c r="S28" s="21"/>
+      <x:c r="S28"/>
     </x:row>
     <x:row r="29" ht="24" customHeight="1">
       <x:c r="A29" s="24"/>
@@ -1179,7 +1203,7 @@
       <x:c r="P29" s="27"/>
       <x:c r="Q29" s="27"/>
       <x:c r="R29" s="33"/>
-      <x:c r="S29" s="21"/>
+      <x:c r="S29"/>
     </x:row>
     <x:row r="30" ht="24" customHeight="1">
       <x:c r="A30" s="24"/>
@@ -1200,7 +1224,7 @@
       <x:c r="P30" s="27"/>
       <x:c r="Q30" s="27"/>
       <x:c r="R30" s="33"/>
-      <x:c r="S30" s="21"/>
+      <x:c r="S30"/>
     </x:row>
     <x:row r="31" ht="24" customHeight="1">
       <x:c r="A31" s="24"/>
@@ -1221,7 +1245,7 @@
       <x:c r="P31" s="27"/>
       <x:c r="Q31" s="27"/>
       <x:c r="R31" s="33"/>
-      <x:c r="S31" s="21"/>
+      <x:c r="S31"/>
     </x:row>
     <x:row r="32" ht="24" customHeight="1">
       <x:c r="A32" s="24"/>
@@ -1242,7 +1266,7 @@
       <x:c r="P32" s="27"/>
       <x:c r="Q32" s="27"/>
       <x:c r="R32" s="33"/>
-      <x:c r="S32" s="21"/>
+      <x:c r="S32"/>
     </x:row>
     <x:row r="33" ht="24" customHeight="1">
       <x:c r="A33" s="24"/>
@@ -1263,7 +1287,7 @@
       <x:c r="P33" s="27"/>
       <x:c r="Q33" s="27"/>
       <x:c r="R33" s="33"/>
-      <x:c r="S33" s="21"/>
+      <x:c r="S33"/>
     </x:row>
     <x:row r="34" ht="24" customHeight="1">
       <x:c r="A34" s="24"/>
@@ -1284,7 +1308,7 @@
       <x:c r="P34" s="27"/>
       <x:c r="Q34" s="27"/>
       <x:c r="R34" s="33"/>
-      <x:c r="S34" s="21"/>
+      <x:c r="S34"/>
     </x:row>
     <x:row r="35" ht="24" customHeight="1">
       <x:c r="A35" s="24"/>
@@ -1305,7 +1329,7 @@
       <x:c r="P35" s="27"/>
       <x:c r="Q35" s="27"/>
       <x:c r="R35" s="33"/>
-      <x:c r="S35" s="21"/>
+      <x:c r="S35"/>
     </x:row>
     <x:row r="36" ht="24" customHeight="1">
       <x:c r="A36" s="24"/>
@@ -1326,7 +1350,7 @@
       <x:c r="P36" s="27"/>
       <x:c r="Q36" s="27"/>
       <x:c r="R36" s="33"/>
-      <x:c r="S36" s="21"/>
+      <x:c r="S36"/>
     </x:row>
     <x:row r="37" ht="24" customHeight="1">
       <x:c r="A37" s="24"/>
@@ -1347,7 +1371,7 @@
       <x:c r="P37" s="27"/>
       <x:c r="Q37" s="27"/>
       <x:c r="R37" s="33"/>
-      <x:c r="S37" s="21"/>
+      <x:c r="S37"/>
     </x:row>
     <x:row r="38" ht="24" customHeight="1">
       <x:c r="A38" s="24"/>
@@ -1368,7 +1392,7 @@
       <x:c r="P38" s="27"/>
       <x:c r="Q38" s="27"/>
       <x:c r="R38" s="33"/>
-      <x:c r="S38" s="21"/>
+      <x:c r="S38"/>
     </x:row>
     <x:row r="39" ht="24" customHeight="1">
       <x:c r="A39" s="24"/>
@@ -1389,7 +1413,7 @@
       <x:c r="P39" s="27"/>
       <x:c r="Q39" s="27"/>
       <x:c r="R39" s="33"/>
-      <x:c r="S39" s="21"/>
+      <x:c r="S39"/>
     </x:row>
     <x:row r="40" ht="24" customHeight="1">
       <x:c r="A40" s="24"/>
@@ -1410,7 +1434,7 @@
       <x:c r="P40" s="27"/>
       <x:c r="Q40" s="27"/>
       <x:c r="R40" s="33"/>
-      <x:c r="S40" s="21"/>
+      <x:c r="S40"/>
     </x:row>
     <x:row r="41" ht="24" customHeight="1">
       <x:c r="A41" s="24"/>
@@ -1431,7 +1455,7 @@
       <x:c r="P41" s="27"/>
       <x:c r="Q41" s="27"/>
       <x:c r="R41" s="33"/>
-      <x:c r="S41" s="21"/>
+      <x:c r="S41"/>
     </x:row>
     <x:row r="42" ht="24" customHeight="1">
       <x:c r="A42" s="24"/>
@@ -1452,7 +1476,7 @@
       <x:c r="P42" s="27"/>
       <x:c r="Q42" s="27"/>
       <x:c r="R42" s="33"/>
-      <x:c r="S42" s="21"/>
+      <x:c r="S42"/>
     </x:row>
     <x:row r="43" ht="24" customHeight="1">
       <x:c r="A43" s="24"/>
@@ -1473,7 +1497,7 @@
       <x:c r="P43" s="27"/>
       <x:c r="Q43" s="27"/>
       <x:c r="R43" s="33"/>
-      <x:c r="S43" s="21"/>
+      <x:c r="S43"/>
     </x:row>
     <x:row r="44" ht="24" customHeight="1">
       <x:c r="A44" s="24"/>
@@ -1494,7 +1518,7 @@
       <x:c r="P44" s="27"/>
       <x:c r="Q44" s="27"/>
       <x:c r="R44" s="33"/>
-      <x:c r="S44" s="21"/>
+      <x:c r="S44"/>
     </x:row>
     <x:row r="45" ht="24" customHeight="1">
       <x:c r="A45" s="24"/>
@@ -1515,7 +1539,7 @@
       <x:c r="P45" s="27"/>
       <x:c r="Q45" s="27"/>
       <x:c r="R45" s="33"/>
-      <x:c r="S45" s="21"/>
+      <x:c r="S45"/>
     </x:row>
     <x:row r="46" ht="24" customHeight="1">
       <x:c r="A46" s="24"/>
@@ -1536,7 +1560,7 @@
       <x:c r="P46" s="27"/>
       <x:c r="Q46" s="27"/>
       <x:c r="R46" s="33"/>
-      <x:c r="S46" s="21"/>
+      <x:c r="S46"/>
     </x:row>
     <x:row r="47" ht="24" customHeight="1">
       <x:c r="A47" s="24"/>
@@ -1557,7 +1581,7 @@
       <x:c r="P47" s="27"/>
       <x:c r="Q47" s="27"/>
       <x:c r="R47" s="33"/>
-      <x:c r="S47" s="21"/>
+      <x:c r="S47"/>
     </x:row>
     <x:row r="48" ht="24" customHeight="1">
       <x:c r="A48" s="24"/>
@@ -1578,7 +1602,7 @@
       <x:c r="P48" s="27"/>
       <x:c r="Q48" s="27"/>
       <x:c r="R48" s="33"/>
-      <x:c r="S48" s="21"/>
+      <x:c r="S48"/>
     </x:row>
     <x:row r="49" ht="24" customHeight="1">
       <x:c r="A49" s="24"/>
@@ -1599,7 +1623,7 @@
       <x:c r="P49" s="27"/>
       <x:c r="Q49" s="27"/>
       <x:c r="R49" s="33"/>
-      <x:c r="S49" s="21"/>
+      <x:c r="S49"/>
     </x:row>
     <x:row r="50" ht="24" customHeight="1">
       <x:c r="A50" s="24"/>
@@ -1620,7 +1644,7 @@
       <x:c r="P50" s="27"/>
       <x:c r="Q50" s="27"/>
       <x:c r="R50" s="33"/>
-      <x:c r="S50" s="21"/>
+      <x:c r="S50"/>
     </x:row>
     <x:row r="51" ht="24" customHeight="1">
       <x:c r="A51" s="24"/>
@@ -1641,7 +1665,7 @@
       <x:c r="P51" s="27"/>
       <x:c r="Q51" s="27"/>
       <x:c r="R51" s="33"/>
-      <x:c r="S51" s="21"/>
+      <x:c r="S51"/>
     </x:row>
     <x:row r="52" ht="24" customHeight="1">
       <x:c r="A52" s="24"/>
@@ -1662,7 +1686,7 @@
       <x:c r="P52" s="27"/>
       <x:c r="Q52" s="27"/>
       <x:c r="R52" s="33"/>
-      <x:c r="S52" s="21"/>
+      <x:c r="S52"/>
     </x:row>
     <x:row r="53" ht="24" customHeight="1">
       <x:c r="A53" s="24"/>
@@ -1683,7 +1707,7 @@
       <x:c r="P53" s="27"/>
       <x:c r="Q53" s="27"/>
       <x:c r="R53" s="33"/>
-      <x:c r="S53" s="21"/>
+      <x:c r="S53"/>
     </x:row>
     <x:row r="54" ht="24" customHeight="1">
       <x:c r="A54" s="24"/>
@@ -1704,7 +1728,7 @@
       <x:c r="P54" s="27"/>
       <x:c r="Q54" s="27"/>
       <x:c r="R54" s="33"/>
-      <x:c r="S54" s="21"/>
+      <x:c r="S54"/>
     </x:row>
     <x:row r="55" ht="24" customHeight="1">
       <x:c r="A55" s="24"/>
@@ -1725,7 +1749,7 @@
       <x:c r="P55" s="27"/>
       <x:c r="Q55" s="27"/>
       <x:c r="R55" s="33"/>
-      <x:c r="S55" s="21"/>
+      <x:c r="S55"/>
     </x:row>
     <x:row r="56" ht="24" customHeight="1">
       <x:c r="A56" s="24"/>
@@ -1746,7 +1770,7 @@
       <x:c r="P56" s="27"/>
       <x:c r="Q56" s="27"/>
       <x:c r="R56" s="33"/>
-      <x:c r="S56" s="21"/>
+      <x:c r="S56"/>
     </x:row>
     <x:row r="57" ht="24" customHeight="1">
       <x:c r="A57" s="24"/>
@@ -1767,7 +1791,7 @@
       <x:c r="P57" s="27"/>
       <x:c r="Q57" s="27"/>
       <x:c r="R57" s="33"/>
-      <x:c r="S57" s="21"/>
+      <x:c r="S57"/>
     </x:row>
     <x:row r="58" ht="24" customHeight="1">
       <x:c r="A58" s="24"/>
@@ -1788,7 +1812,7 @@
       <x:c r="P58" s="27"/>
       <x:c r="Q58" s="27"/>
       <x:c r="R58" s="33"/>
-      <x:c r="S58" s="21"/>
+      <x:c r="S58"/>
     </x:row>
     <x:row r="59" ht="24" customHeight="1">
       <x:c r="A59" s="24"/>
@@ -1809,7 +1833,7 @@
       <x:c r="P59" s="27"/>
       <x:c r="Q59" s="27"/>
       <x:c r="R59" s="33"/>
-      <x:c r="S59" s="21"/>
+      <x:c r="S59"/>
     </x:row>
     <x:row r="60" ht="24" customHeight="1">
       <x:c r="A60" s="24"/>
@@ -1830,7 +1854,7 @@
       <x:c r="P60" s="27"/>
       <x:c r="Q60" s="27"/>
       <x:c r="R60" s="33"/>
-      <x:c r="S60" s="21"/>
+      <x:c r="S60"/>
     </x:row>
     <x:row r="61" ht="24" customHeight="1">
       <x:c r="A61" s="24"/>
@@ -1851,7 +1875,7 @@
       <x:c r="P61" s="27"/>
       <x:c r="Q61" s="27"/>
       <x:c r="R61" s="33"/>
-      <x:c r="S61" s="21"/>
+      <x:c r="S61"/>
     </x:row>
     <x:row r="62" ht="24" customHeight="1">
       <x:c r="A62" s="24"/>
@@ -1872,7 +1896,7 @@
       <x:c r="P62" s="27"/>
       <x:c r="Q62" s="27"/>
       <x:c r="R62" s="33"/>
-      <x:c r="S62" s="21"/>
+      <x:c r="S62"/>
     </x:row>
     <x:row r="63" ht="24" customHeight="1">
       <x:c r="A63" s="24"/>
@@ -1893,7 +1917,7 @@
       <x:c r="P63" s="27"/>
       <x:c r="Q63" s="27"/>
       <x:c r="R63" s="33"/>
-      <x:c r="S63" s="21"/>
+      <x:c r="S63"/>
     </x:row>
     <x:row r="64" ht="24" customHeight="1">
       <x:c r="A64" s="24"/>
@@ -1914,7 +1938,7 @@
       <x:c r="P64" s="27"/>
       <x:c r="Q64" s="27"/>
       <x:c r="R64" s="33"/>
-      <x:c r="S64" s="21"/>
+      <x:c r="S64"/>
     </x:row>
     <x:row r="65" ht="24" customHeight="1">
       <x:c r="A65" s="24"/>
@@ -1935,7 +1959,7 @@
       <x:c r="P65" s="27"/>
       <x:c r="Q65" s="27"/>
       <x:c r="R65" s="33"/>
-      <x:c r="S65" s="21"/>
+      <x:c r="S65"/>
     </x:row>
     <x:row r="66" ht="24" customHeight="1">
       <x:c r="A66" s="24"/>
@@ -1956,7 +1980,7 @@
       <x:c r="P66" s="27"/>
       <x:c r="Q66" s="27"/>
       <x:c r="R66" s="33"/>
-      <x:c r="S66" s="21"/>
+      <x:c r="S66"/>
     </x:row>
     <x:row r="67" ht="24" customHeight="1">
       <x:c r="A67" s="24"/>
@@ -1977,7 +2001,7 @@
       <x:c r="P67" s="27"/>
       <x:c r="Q67" s="27"/>
       <x:c r="R67" s="33"/>
-      <x:c r="S67" s="21"/>
+      <x:c r="S67"/>
     </x:row>
     <x:row r="68" ht="24" customHeight="1">
       <x:c r="A68" s="24"/>
@@ -1998,7 +2022,7 @@
       <x:c r="P68" s="27"/>
       <x:c r="Q68" s="27"/>
       <x:c r="R68" s="33"/>
-      <x:c r="S68" s="21"/>
+      <x:c r="S68"/>
     </x:row>
     <x:row r="69" ht="24" customHeight="1">
       <x:c r="A69" s="24"/>
@@ -2019,7 +2043,7 @@
       <x:c r="P69" s="27"/>
       <x:c r="Q69" s="27"/>
       <x:c r="R69" s="33"/>
-      <x:c r="S69" s="21"/>
+      <x:c r="S69"/>
     </x:row>
     <x:row r="70" ht="24" customHeight="1">
       <x:c r="A70" s="24"/>
@@ -2040,7 +2064,7 @@
       <x:c r="P70" s="27"/>
       <x:c r="Q70" s="27"/>
       <x:c r="R70" s="33"/>
-      <x:c r="S70" s="21"/>
+      <x:c r="S70"/>
     </x:row>
     <x:row r="71" ht="24" customHeight="1">
       <x:c r="A71" s="24"/>
@@ -2061,7 +2085,7 @@
       <x:c r="P71" s="27"/>
       <x:c r="Q71" s="27"/>
       <x:c r="R71" s="33"/>
-      <x:c r="S71" s="21"/>
+      <x:c r="S71"/>
     </x:row>
     <x:row r="72" ht="24" customHeight="1">
       <x:c r="A72" s="24"/>
@@ -2082,7 +2106,7 @@
       <x:c r="P72" s="27"/>
       <x:c r="Q72" s="27"/>
       <x:c r="R72" s="33"/>
-      <x:c r="S72" s="21"/>
+      <x:c r="S72"/>
     </x:row>
     <x:row r="73" ht="24" customHeight="1">
       <x:c r="A73" s="24"/>
@@ -2103,7 +2127,7 @@
       <x:c r="P73" s="27"/>
       <x:c r="Q73" s="27"/>
       <x:c r="R73" s="33"/>
-      <x:c r="S73" s="21"/>
+      <x:c r="S73"/>
     </x:row>
     <x:row r="74" ht="24" customHeight="1">
       <x:c r="A74" s="24"/>
@@ -2124,7 +2148,7 @@
       <x:c r="P74" s="27"/>
       <x:c r="Q74" s="27"/>
       <x:c r="R74" s="33"/>
-      <x:c r="S74" s="21"/>
+      <x:c r="S74"/>
     </x:row>
     <x:row r="75" ht="24" customHeight="1">
       <x:c r="A75" s="24"/>
@@ -2145,7 +2169,7 @@
       <x:c r="P75" s="27"/>
       <x:c r="Q75" s="27"/>
       <x:c r="R75" s="33"/>
-      <x:c r="S75" s="21"/>
+      <x:c r="S75"/>
     </x:row>
     <x:row r="76" ht="24" customHeight="1">
       <x:c r="A76" s="24"/>
@@ -2166,7 +2190,7 @@
       <x:c r="P76" s="27"/>
       <x:c r="Q76" s="27"/>
       <x:c r="R76" s="33"/>
-      <x:c r="S76" s="21"/>
+      <x:c r="S76"/>
     </x:row>
     <x:row r="77" ht="24" customHeight="1">
       <x:c r="A77" s="24"/>
@@ -2187,7 +2211,7 @@
       <x:c r="P77" s="27"/>
       <x:c r="Q77" s="27"/>
       <x:c r="R77" s="33"/>
-      <x:c r="S77" s="21"/>
+      <x:c r="S77"/>
     </x:row>
     <x:row r="78" ht="24" customHeight="1">
       <x:c r="A78" s="24"/>
@@ -2208,7 +2232,7 @@
       <x:c r="P78" s="27"/>
       <x:c r="Q78" s="27"/>
       <x:c r="R78" s="33"/>
-      <x:c r="S78" s="21"/>
+      <x:c r="S78"/>
     </x:row>
     <x:row r="79" ht="24" customHeight="1">
       <x:c r="A79" s="24"/>
@@ -2229,7 +2253,7 @@
       <x:c r="P79" s="27"/>
       <x:c r="Q79" s="27"/>
       <x:c r="R79" s="33"/>
-      <x:c r="S79" s="21"/>
+      <x:c r="S79"/>
     </x:row>
     <x:row r="80" ht="24" customHeight="1">
       <x:c r="A80" s="24"/>
@@ -2250,7 +2274,7 @@
       <x:c r="P80" s="27"/>
       <x:c r="Q80" s="27"/>
       <x:c r="R80" s="33"/>
-      <x:c r="S80" s="21"/>
+      <x:c r="S80"/>
     </x:row>
     <x:row r="81" ht="24" customHeight="1">
       <x:c r="A81" s="24"/>
@@ -2271,7 +2295,7 @@
       <x:c r="P81" s="27"/>
       <x:c r="Q81" s="27"/>
       <x:c r="R81" s="33"/>
-      <x:c r="S81" s="21"/>
+      <x:c r="S81"/>
     </x:row>
     <x:row r="82" ht="24" customHeight="1">
       <x:c r="A82" s="24"/>
@@ -2292,7 +2316,7 @@
       <x:c r="P82" s="27"/>
       <x:c r="Q82" s="27"/>
       <x:c r="R82" s="33"/>
-      <x:c r="S82" s="21"/>
+      <x:c r="S82"/>
     </x:row>
     <x:row r="83" ht="24" customHeight="1">
       <x:c r="A83" s="24"/>
@@ -2313,7 +2337,7 @@
       <x:c r="P83" s="27"/>
       <x:c r="Q83" s="27"/>
       <x:c r="R83" s="33"/>
-      <x:c r="S83" s="21"/>
+      <x:c r="S83"/>
     </x:row>
     <x:row r="84" ht="24" customHeight="1">
       <x:c r="A84" s="24"/>
@@ -2334,7 +2358,7 @@
       <x:c r="P84" s="27"/>
       <x:c r="Q84" s="27"/>
       <x:c r="R84" s="33"/>
-      <x:c r="S84" s="21"/>
+      <x:c r="S84"/>
     </x:row>
     <x:row r="85" ht="24" customHeight="1">
       <x:c r="A85" s="24"/>
@@ -2355,7 +2379,7 @@
       <x:c r="P85" s="27"/>
       <x:c r="Q85" s="27"/>
       <x:c r="R85" s="33"/>
-      <x:c r="S85" s="21"/>
+      <x:c r="S85"/>
     </x:row>
     <x:row r="86" ht="24" customHeight="1">
       <x:c r="A86" s="24"/>
@@ -2376,7 +2400,7 @@
       <x:c r="P86" s="27"/>
       <x:c r="Q86" s="27"/>
       <x:c r="R86" s="33"/>
-      <x:c r="S86" s="21"/>
+      <x:c r="S86"/>
     </x:row>
     <x:row r="87" ht="24" customHeight="1">
       <x:c r="A87" s="24"/>
@@ -2397,7 +2421,7 @@
       <x:c r="P87" s="27"/>
       <x:c r="Q87" s="27"/>
       <x:c r="R87" s="33"/>
-      <x:c r="S87" s="21"/>
+      <x:c r="S87"/>
     </x:row>
     <x:row r="88" ht="24" customHeight="1">
       <x:c r="A88" s="24"/>
@@ -2418,7 +2442,7 @@
       <x:c r="P88" s="27"/>
       <x:c r="Q88" s="27"/>
       <x:c r="R88" s="33"/>
-      <x:c r="S88" s="21"/>
+      <x:c r="S88"/>
     </x:row>
     <x:row r="89" ht="24" customHeight="1">
       <x:c r="A89" s="24"/>
@@ -2439,7 +2463,7 @@
       <x:c r="P89" s="27"/>
       <x:c r="Q89" s="27"/>
       <x:c r="R89" s="33"/>
-      <x:c r="S89" s="21"/>
+      <x:c r="S89"/>
     </x:row>
     <x:row r="90" ht="24" customHeight="1">
       <x:c r="A90" s="24"/>
@@ -2460,7 +2484,7 @@
       <x:c r="P90" s="27"/>
       <x:c r="Q90" s="27"/>
       <x:c r="R90" s="33"/>
-      <x:c r="S90" s="21"/>
+      <x:c r="S90"/>
     </x:row>
     <x:row r="91" ht="24" customHeight="1">
       <x:c r="A91" s="24"/>
@@ -2481,7 +2505,7 @@
       <x:c r="P91" s="27"/>
       <x:c r="Q91" s="27"/>
       <x:c r="R91" s="33"/>
-      <x:c r="S91" s="21"/>
+      <x:c r="S91"/>
     </x:row>
     <x:row r="92" ht="24" customHeight="1">
       <x:c r="A92" s="24"/>
@@ -2502,7 +2526,7 @@
       <x:c r="P92" s="27"/>
       <x:c r="Q92" s="27"/>
       <x:c r="R92" s="33"/>
-      <x:c r="S92" s="21"/>
+      <x:c r="S92"/>
     </x:row>
     <x:row r="93" ht="24" customHeight="1">
       <x:c r="A93" s="24"/>
@@ -2523,7 +2547,7 @@
       <x:c r="P93" s="27"/>
       <x:c r="Q93" s="27"/>
       <x:c r="R93" s="33"/>
-      <x:c r="S93" s="21"/>
+      <x:c r="S93"/>
     </x:row>
     <x:row r="94" ht="24" customHeight="1">
       <x:c r="A94" s="24"/>
@@ -2544,7 +2568,7 @@
       <x:c r="P94" s="27"/>
       <x:c r="Q94" s="27"/>
       <x:c r="R94" s="33"/>
-      <x:c r="S94" s="21"/>
+      <x:c r="S94"/>
     </x:row>
     <x:row r="95" ht="24" customHeight="1">
       <x:c r="A95" s="24"/>
@@ -2565,7 +2589,7 @@
       <x:c r="P95" s="27"/>
       <x:c r="Q95" s="27"/>
       <x:c r="R95" s="33"/>
-      <x:c r="S95" s="21"/>
+      <x:c r="S95"/>
     </x:row>
     <x:row r="96" ht="24" customHeight="1">
       <x:c r="A96" s="24"/>
@@ -2586,7 +2610,7 @@
       <x:c r="P96" s="27"/>
       <x:c r="Q96" s="27"/>
       <x:c r="R96" s="33"/>
-      <x:c r="S96" s="21"/>
+      <x:c r="S96"/>
     </x:row>
     <x:row r="97" ht="24" customHeight="1">
       <x:c r="A97" s="24"/>
@@ -2607,7 +2631,7 @@
       <x:c r="P97" s="27"/>
       <x:c r="Q97" s="27"/>
       <x:c r="R97" s="33"/>
-      <x:c r="S97" s="21"/>
+      <x:c r="S97"/>
     </x:row>
     <x:row r="98" ht="24" customHeight="1">
       <x:c r="A98" s="24"/>
@@ -2628,7 +2652,7 @@
       <x:c r="P98" s="27"/>
       <x:c r="Q98" s="27"/>
       <x:c r="R98" s="33"/>
-      <x:c r="S98" s="21"/>
+      <x:c r="S98"/>
     </x:row>
     <x:row r="99" ht="24" customHeight="1">
       <x:c r="A99" s="24"/>
@@ -2649,7 +2673,7 @@
       <x:c r="P99" s="27"/>
       <x:c r="Q99" s="27"/>
       <x:c r="R99" s="33"/>
-      <x:c r="S99" s="21"/>
+      <x:c r="S99"/>
     </x:row>
     <x:row r="100" ht="24" customHeight="1">
       <x:c r="A100" s="24"/>
@@ -2670,7 +2694,7 @@
       <x:c r="P100" s="27"/>
       <x:c r="Q100" s="27"/>
       <x:c r="R100" s="33"/>
-      <x:c r="S100" s="21"/>
+      <x:c r="S100"/>
     </x:row>
     <x:row r="101" ht="24" customHeight="1">
       <x:c r="A101" s="25"/>
@@ -2691,7 +2715,7 @@
       <x:c r="P101" s="28"/>
       <x:c r="Q101" s="28"/>
       <x:c r="R101" s="34"/>
-      <x:c r="S101" s="22"/>
+      <x:c r="S101"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
@@ -2703,6 +2727,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80c0e54b0d4244b0"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -2836,84 +2863,104 @@
     </x:row>
     <x:row r="11" ht="44" customHeight="1">
       <x:c r="A11" s="48" t="str">
-        <x:v>状态</x:v>
+        <x:v>归属部门</x:v>
       </x:c>
       <x:c r="B11" s="48" t="str">
-        <x:v>可填写在库、借用中、使用中、报废，或设置中新增的状态名称；留空默认为在库。</x:v>
+        <x:v>无需填写。系统会按责任人的员工档案自动带出；未填写责任人时部门保持为空。</x:v>
       </x:c>
       <x:c r="C11" s="48" t="str">
         <x:v>否</x:v>
       </x:c>
       <x:c r="D11" s="48" t="str">
-        <x:v>在库</x:v>
+        <x:v>自动带出</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="44" customHeight="1">
       <x:c r="A12" s="48" t="str">
-        <x:v>品牌和型号</x:v>
+        <x:v>状态</x:v>
       </x:c>
       <x:c r="B12" s="48" t="str">
-        <x:v>建议分别填写，系统会据此生成资产显示名称。</x:v>
+        <x:v>可填写在库、借用中、使用中、报废，或设置中新增的状态名称；留空默认为在库。</x:v>
       </x:c>
       <x:c r="C12" s="48" t="str">
-        <x:v>建议</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="D12" s="48" t="str">
-        <x:v>Lenovo / ThinkBook 14</x:v>
+        <x:v>在库</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="44" customHeight="1">
       <x:c r="A13" s="48" t="str">
-        <x:v>数量</x:v>
+        <x:v>品牌和型号</x:v>
       </x:c>
       <x:c r="B13" s="48" t="str">
-        <x:v>资产按一物一码管理，每行固定填写 1。</x:v>
+        <x:v>建议分别填写，系统会据此生成资产显示名称。</x:v>
       </x:c>
       <x:c r="C13" s="48" t="str">
-        <x:v>是</x:v>
-      </x:c>
-      <x:c r="D13" s="53" t="n">
-        <x:v>1</x:v>
+        <x:v>建议</x:v>
+      </x:c>
+      <x:c r="D13" s="53" t="str">
+        <x:v>Lenovo / ThinkBook 14</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="44" customHeight="1">
       <x:c r="A14" s="48" t="str">
-        <x:v>日期</x:v>
+        <x:v>数量</x:v>
       </x:c>
       <x:c r="B14" s="48" t="str">
-        <x:v>请使用 yyyy-mm-dd 格式。</x:v>
+        <x:v>资产按一物一码管理，每行固定填写 1。</x:v>
       </x:c>
       <x:c r="C14" s="48" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="D14" s="48" t="str">
-        <x:v>2026-07-28</x:v>
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="D14" s="48" t="n">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="44" customHeight="1">
       <x:c r="A15" s="48" t="str">
+        <x:v>日期</x:v>
+      </x:c>
+      <x:c r="B15" s="48" t="str">
+        <x:v>请使用 yyyy-mm-dd 格式。</x:v>
+      </x:c>
+      <x:c r="C15" s="48" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="D15" s="48" t="str">
+        <x:v>2026-07-28</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
         <x:v>导入规则</x:v>
       </x:c>
-      <x:c r="B15" s="48" t="str">
+      <x:c r="B16" t="str">
         <x:v>系统会先预检整批数据；只有阻止性错误需要先修正，提示项可先导入后再完善。</x:v>
       </x:c>
-      <x:c r="C15" s="48" t="str">
+      <x:c r="C16" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="D15" s="48" t="str"/>
+      <x:c r="D16"/>
     </x:row>
     <x:row r="17" ht="38" customHeight="1">
-      <x:c r="A17" s="52" t="str">
-        <x:v>注意：请不要删除或改名第 1 行表头；需要更多行时可继续向下填写。</x:v>
-      </x:c>
+      <x:c r="A17" s="52"/>
       <x:c r="B17" s="52"/>
       <x:c r="C17" s="52"/>
       <x:c r="D17" s="52"/>
     </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>注意：请不要删除或改名第 1 行表头；需要更多行时可继续向下填写。</x:v>
+      </x:c>
+      <x:c r="B18"/>
+      <x:c r="C18"/>
+      <x:c r="D18"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>
-    <x:mergeCell ref="A17:D17"/>
+    <x:mergeCell ref="A18:D18"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>